<commit_message>
Add BigQuery sheet, optional service section, and cost bar chart
변경 사항:
- BigQuery 세부 견적 시트 추가 (Sheet5b)
  - 사용 여부 토글(예/아니오)로 비용 자동 ON/OFF
  - 스토리지($0.023/GB) + 온디맨드 쿼리($6.25/TB) 계산
  - VLOOKUP으로 단가표 참조

- Sheet1 고객 입력에 선택 서비스 섹션 추가
  - BigQuery 사용 여부 (드롭다운)
  - BigQuery 저장 데이터(GB) / 월 쿼리 스캔량(TB) 입력

- Sheet6 최종 견적 요약 개선
  - 선택 서비스(Optional) 섹션 추가 (Row 21~24)
  - 전체 합계(필수+선택) 행 추가 (Row 26)
  - 서비스별 월 비용 분포 BarChart 삽입 (H2, Google Blue)

- Sheet7 단가표에 BigQuery 단가 추가 (Row 22~23)

https://claude.ai/code/session_01CTM9sBCyfMDDfHkCAxJL2n
</commit_message>
<xml_diff>
--- a/gcp_estimate.xlsx
+++ b/gcp_estimate.xlsx
@@ -12,8 +12,9 @@
     <sheet name="Cloud Storage 세부 견적" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Cloud SQL 세부 견적" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Networking 세부 견적" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="최종 견적 요약" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="단가표" sheetId="7" state="hidden" r:id="rId7"/>
+    <sheet name="BigQuery 세부 견적" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="최종 견적 요약" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="단가표" sheetId="8" state="hidden" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="EXCHANGE_RATE">'고객 입력'!$B$3</definedName>
@@ -28,7 +29,7 @@
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="&quot;₩&quot;#,##0"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -79,8 +80,21 @@
       <color rgb="005F6368"/>
       <sz val="9"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="007B1FA2"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00137333"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -123,6 +137,24 @@
         <bgColor rgb="00E6F4EA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F3E5F5"/>
+        <bgColor rgb="00F3E5F5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00CE93D8"/>
+        <bgColor rgb="00CE93D8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E1BEE7"/>
+        <bgColor rgb="00E1BEE7"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -142,7 +174,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -200,6 +232,20 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="13" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -284,6 +330,152 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>서비스별 월 비용 분포 (On-Demand, USD)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'최종 견적 요약'!E5</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="4285F4"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="2962FF"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'최종 견적 요약'!$A$6:$A$9</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'최종 견적 요약'!$E$6:$E$9</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>서비스</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>월 비용 (USD)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7920000" cy="5040000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -575,7 +767,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -771,9 +963,49 @@
         <v>1000</v>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>▶  선택 서비스 (Optional)</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>BigQuery 사용 여부</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>아니오</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>BigQuery 저장 데이터 (GB)</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>BigQuery 월 쿼리 스캔량 (TB)</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
-  <dataValidations count="8">
+  <dataValidations count="9">
     <dataValidation sqref="B4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"asia-northeast3,asia-northeast1,asia-east1,us-central1"</formula1>
     </dataValidation>
@@ -789,13 +1021,16 @@
     <dataValidation sqref="B13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"소형,중형,대형"</formula1>
     </dataValidation>
-    <dataValidation sqref="B14 B17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="B14 B17 B20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"예,아니오"</formula1>
     </dataValidation>
     <dataValidation sqref="B15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"무료 PostgreSQL,MS SQL"</formula1>
     </dataValidation>
-    <dataValidation sqref="B14 B17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="B14 B17 B20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"예,아니오"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B14 B17 B20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"예,아니오"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1193,7 +1428,103 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>항목</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>값 / 수식</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>BigQuery 사용 여부</t>
+        </is>
+      </c>
+      <c r="B2" s="8">
+        <f>'고객 입력'!B20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>저장 데이터 (GB)</t>
+        </is>
+      </c>
+      <c r="B3" s="8">
+        <f>'고객 입력'!B21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>월 쿼리 스캔량 (TB)</t>
+        </is>
+      </c>
+      <c r="B4" s="8">
+        <f>'고객 입력'!B22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>스토리지 단가 ($/GB)</t>
+        </is>
+      </c>
+      <c r="B5" s="8">
+        <f>VLOOKUP("BQ Storage Active", 단가표!$A$22:$B$23, 2, FALSE)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>쿼리 단가 ($/TB)</t>
+        </is>
+      </c>
+      <c r="B6" s="8">
+        <f>VLOOKUP("BQ Query ($/TB)", 단가표!$A$22:$B$23, 2, FALSE)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>월 합계 (USD)</t>
+        </is>
+      </c>
+      <c r="B7" s="9">
+        <f>IF(B2="예", B3*B5 + B4*B6, 0)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1506,12 +1837,119 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="26" t="inlineStr">
+        <is>
+          <t>선택 서비스 (Optional Services)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="27" t="inlineStr">
+        <is>
+          <t>서비스명 (GCP)</t>
+        </is>
+      </c>
+      <c r="B22" s="27" t="inlineStr">
+        <is>
+          <t>스펙 / 상세</t>
+        </is>
+      </c>
+      <c r="C22" s="27" t="inlineStr">
+        <is>
+          <t>수량</t>
+        </is>
+      </c>
+      <c r="D22" s="27" t="inlineStr">
+        <is>
+          <t>시간당 단가 (USD)</t>
+        </is>
+      </c>
+      <c r="E22" s="27" t="inlineStr">
+        <is>
+          <t>월 비용 (USD)</t>
+        </is>
+      </c>
+      <c r="F22" s="27" t="inlineStr">
+        <is>
+          <t>월 비용 (KRW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>BigQuery</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>Storage + On-Demand Query</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>1 식</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E23" s="9">
+        <f>'BigQuery 세부 견적'!B7</f>
+        <v/>
+      </c>
+      <c r="F23" s="20">
+        <f>E23*EXCHANGE_RATE</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="28" t="inlineStr">
+        <is>
+          <t>선택 서비스 소계</t>
+        </is>
+      </c>
+      <c r="B24" s="28" t="inlineStr"/>
+      <c r="C24" s="28" t="inlineStr"/>
+      <c r="D24" s="28" t="inlineStr"/>
+      <c r="E24" s="29">
+        <f>E23</f>
+        <v/>
+      </c>
+      <c r="F24" s="30">
+        <f>F23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="31" t="inlineStr">
+        <is>
+          <t>전체 합계 (필수 + 선택 서비스, 종량제 기준)</t>
+        </is>
+      </c>
+      <c r="B26" s="22" t="n"/>
+      <c r="C26" s="22" t="n"/>
+      <c r="D26" s="22" t="n"/>
+      <c r="E26" s="32">
+        <f>E10+E24</f>
+        <v/>
+      </c>
+      <c r="F26" s="33">
+        <f>F10+F24</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="6">
+    <mergeCell ref="A17:D17"/>
     <mergeCell ref="A19:F19"/>
-    <mergeCell ref="A17:D17"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A26:D26"/>
     <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A21:F21"/>
   </mergeCells>
   <conditionalFormatting sqref="E6:E9">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
@@ -1519,16 +1957,17 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1536,29 +1975,29 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="26" t="inlineStr">
+      <c r="A1" s="34" t="inlineStr">
         <is>
           <t>[Compute Engine] — asia-northeast3 기준 On-Demand (USD/시간)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="27" t="inlineStr">
+      <c r="A2" s="35" t="inlineStr">
         <is>
           <t>규모</t>
         </is>
       </c>
-      <c r="B2" s="27" t="inlineStr">
+      <c r="B2" s="35" t="inlineStr">
         <is>
           <t>스펙</t>
         </is>
       </c>
-      <c r="C2" s="27" t="inlineStr">
+      <c r="C2" s="35" t="inlineStr">
         <is>
           <t>Linux단가</t>
         </is>
       </c>
-      <c r="D2" s="27" t="inlineStr">
+      <c r="D2" s="35" t="inlineStr">
         <is>
           <t>Windows추가단가</t>
         </is>
@@ -1637,29 +2076,29 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="26" t="inlineStr">
+      <c r="A8" s="34" t="inlineStr">
         <is>
           <t>[Cloud SQL] — asia-northeast3 기준 On-Demand (USD/시간)</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="27" t="inlineStr">
+      <c r="A9" s="35" t="inlineStr">
         <is>
           <t>규모</t>
         </is>
       </c>
-      <c r="B9" s="27" t="inlineStr">
+      <c r="B9" s="35" t="inlineStr">
         <is>
           <t>스펙</t>
         </is>
       </c>
-      <c r="C9" s="27" t="inlineStr">
+      <c r="C9" s="35" t="inlineStr">
         <is>
           <t>Base단가</t>
         </is>
       </c>
-      <c r="D9" s="27" t="inlineStr">
+      <c r="D9" s="35" t="inlineStr">
         <is>
           <t>MSSQL추가단가</t>
         </is>
@@ -1720,25 +2159,25 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="26" t="inlineStr">
+      <c r="A14" s="34" t="inlineStr">
         <is>
           <t>[기타 서비스] — USD 단가</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="27" t="inlineStr">
+      <c r="A15" s="35" t="inlineStr">
         <is>
           <t>항목</t>
         </is>
       </c>
-      <c r="B15" s="27" t="inlineStr">
+      <c r="B15" s="35" t="inlineStr">
         <is>
           <t>단가</t>
         </is>
       </c>
-      <c r="C15" s="27" t="inlineStr"/>
-      <c r="D15" s="27" t="inlineStr"/>
+      <c r="C15" s="35" t="inlineStr"/>
+      <c r="D15" s="35" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1775,6 +2214,51 @@
       </c>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>[BigQuery] — asia-northeast3 기준 USD 단가</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>항목</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>단가</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>BQ Storage Active</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>BQ Query ($/TB)</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>